<commit_message>
Test case 6& 7
</commit_message>
<xml_diff>
--- a/testdata/Logintestdata.xlsx
+++ b/testdata/Logintestdata.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="13365" windowHeight="11040"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="23055" windowHeight="11220"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,13 +35,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -61,13 +68,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -375,11 +388,14 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="Giri@123"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>